<commit_message>
fix: correct template compliance — AC numbering, US011 actor, sequential IDs, report structure
Monitor debate findings applied:
- Acceptance Criteria: '1)' → '1.' format
- US011: 'system' actor → 'administrator'
- Story IDs: re-sorted to sequential US001-US022
- Report: removed out-of-scope chapters (Risk Assessment, Git Strategy)
- Report: strict 4-chapter structure per template
- Report: Supporting Material properly scoped
- Team info fields marked [TO BE FILLED]
</commit_message>
<xml_diff>
--- a/deliverables/ProductBacklog_group104.xlsx
+++ b/deliverables/ProductBacklog_group104.xlsx
@@ -55,10 +55,10 @@
     <t xml:space="preserve">Sprint 1</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Can enter email and password
-2) Password strength validation
-3) Success confirmation
-4) Email verification link</t>
+    <t xml:space="preserve">1. Can enter email and password
+2. Password strength validation
+3. Success confirmation
+4. Email verification link</t>
   </si>
   <si>
     <t xml:space="preserve">5</t>
@@ -82,15 +82,58 @@
     <t xml:space="preserve">As a registered user, I want to log in, so that I can access my data.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Correct credentials allow login
-2) Wrong password shows error
-3) Remember login state
-4) Redirect to home after login</t>
+    <t xml:space="preserve">1. Correct credentials allow login
+2. Wrong password shows error
+3. Remember login state
+4. Redirect to home after login</t>
   </si>
   <si>
     <t xml:space="preserve">3</t>
   </si>
   <si>
+    <t xml:space="preserve">US003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change Password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to change my password, so that I can keep my account secure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter old and new password
+2. Confirm new password
+3. Success notification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permission Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As an administrator, I want to manage user roles, so that I can control access permissions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Assign user roles
+2. View role list
+3. Modify user permissions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-14</t>
+  </si>
+  <si>
     <t xml:space="preserve">US005</t>
   </si>
   <si>
@@ -100,14 +143,124 @@
     <t xml:space="preserve">As a user, I want to log out, so that I can protect my privacy on shared devices.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Click logout button
-2) Clear session
-3) Redirect to login page</t>
+    <t xml:space="preserve">1. Click logout button
+2. Clear session
+3. Redirect to login page</t>
   </si>
   <si>
     <t xml:space="preserve">2</t>
   </si>
   <si>
+    <t xml:space="preserve">US006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create Record</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to create new data records, so that I can manage my information.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fill in form fields
+2. Save success notification
+3. Auto-generate ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">View Records</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to view existing records, so that I can understand the current status.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. List all records
+2. Click to view details
+3. Pagination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edit Record</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to edit existing records, so that I can update information.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Modify form fields
+2. Save update
+3. Version tracking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delete Record</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to delete unwanted records, so that I can keep data clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Confirmation prompt
+2. Soft delete (recoverable)
+3. Permanent delete option</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batch Operations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As an administrator, I want to batch process data, so that I can improve efficiency.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Select multiple records
+2. Batch delete/edit/export
+3. Operation confirmation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Validation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As an administrator, I want the system to validate input data, so that I can ensure data quality and prevent errors.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Required field check
+2. Format validation
+3. Uniqueness check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Persistence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a system, I want to permanently store data, so that users can access it next time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Database storage
+2. No data loss
+3. Backup support</t>
+  </si>
+  <si>
     <t xml:space="preserve">US013</t>
   </si>
   <si>
@@ -117,14 +270,48 @@
     <t xml:space="preserve">As a user, I want to browse the system via navigation menu, so that I can quickly find features.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Sidebar navigation
-2) Current page highlighted
-3) Responsive menu</t>
+    <t xml:space="preserve">1. Sidebar navigation
+2. Current page highlighted
+3. Responsive menu</t>
   </si>
   <si>
     <t xml:space="preserve">2026-04-09</t>
   </si>
   <si>
+    <t xml:space="preserve">US014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a user, I want to see overview data on a dashboard, so that I can quickly understand the status.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Statistics display
+2. Chart visualisation
+3. Quick action entry points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsive Design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a mobile user, I want to use the system on my phone, so that I can access it anywhere.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Adapt to mobile screens
+2. Touch operation support
+3. Fast loading</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-28</t>
+  </si>
+  <si>
     <t xml:space="preserve">US016</t>
   </si>
   <si>
@@ -134,196 +321,9 @@
     <t xml:space="preserve">As a user, I want to fill in clear forms, so that I can efficiently input data.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Clear labels
-2) Input hint text
-3) Real-time validation feedback</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Change Password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a user, I want to change my password, so that I can keep my account secure.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Should</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Enter old and new password
-2) Confirm new password
-3) Success notification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permission Management</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an administrator, I want to manage user roles, so that I can control access permissions.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Assign user roles
-2) View role list
-3) Modify user permissions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create Record</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a user, I want to create new data records, so that I can manage my information.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Fill in form fields
-2) Save success notification
-3) Auto-generate ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">View Records</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a user, I want to view existing records, so that I can understand the current status.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) List all records
-2) Click to view details
-3) Pagination</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edit Record</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a user, I want to edit existing records, so that I can update information.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Modify form fields
-2) Save update
-3) Version tracking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data Validation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a system, I want to validate input data legality, so that I can prevent errors.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Required field check
-2) Format validation
-3) Uniqueness check</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data Persistence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a system, I want to permanently store data, so that users can access it next time.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Database storage
-2) No data loss
-3) Backup support</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delete Record</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a user, I want to delete unwanted records, so that I can keep data clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Confirmation prompt
-2) Soft delete (recoverable)
-3) Permanent delete option</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Batch Operations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an administrator, I want to batch process data, so that I can improve efficiency.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Could</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Select multiple records
-2) Batch delete/edit/export
-3) Operation confirmation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dashboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a user, I want to see overview data on a dashboard, so that I can quickly understand the status.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Statistics display
-2) Chart visualisation
-3) Quick action entry points</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Responsive Design</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a mobile user, I want to use the system on my phone, so that I can access it anywhere.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) Adapt to mobile screens
-2) Touch operation support
-3) Fast loading</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-28</t>
+    <t xml:space="preserve">1. Clear labels
+2. Input hint text
+3. Real-time validation feedback</t>
   </si>
   <si>
     <t xml:space="preserve">US017</t>
@@ -335,9 +335,9 @@
     <t xml:space="preserve">As a user, I want to receive operation feedback notifications, so that I can understand system status.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Success/failure prompts
-2) Toast messages
-3) Dismissable notifications</t>
+    <t xml:space="preserve">1. Success/failure prompts
+2. Toast messages
+3. Dismissable notifications</t>
   </si>
   <si>
     <t xml:space="preserve">US018</t>
@@ -349,9 +349,9 @@
     <t xml:space="preserve">As a user, I want to search records, so that I can quickly find target data.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Keyword search input
-2) Highlight matching results
-3) Search history</t>
+    <t xml:space="preserve">1. Keyword search input
+2. Highlight matching results
+3. Search history</t>
   </si>
   <si>
     <t xml:space="preserve">2026-05-05</t>
@@ -366,9 +366,9 @@
     <t xml:space="preserve">As a user, I want to filter data by conditions, so that I can precisely select.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Multiple condition combination
-2) Date range filter
-3) Status filter</t>
+    <t xml:space="preserve">1. Multiple condition combination
+2. Date range filter
+3. Status filter</t>
   </si>
   <si>
     <t xml:space="preserve">US020</t>
@@ -380,9 +380,9 @@
     <t xml:space="preserve">As a user, I want to sort records, so that I can view them by priority.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Sort by date
-2) Sort by name
-3) Sort by priority</t>
+    <t xml:space="preserve">1. Sort by date
+2. Sort by name
+3. Sort by priority</t>
   </si>
   <si>
     <t xml:space="preserve">US021</t>
@@ -397,9 +397,9 @@
     <t xml:space="preserve">Sprint 5</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Select export fields
-2) Generate .xlsx file
-3) Auto-download</t>
+    <t xml:space="preserve">1. Select export fields
+2. Generate .xlsx file
+3. Auto-download</t>
   </si>
   <si>
     <t xml:space="preserve">2026-05-12</t>
@@ -414,9 +414,9 @@
     <t xml:space="preserve">As an administrator, I want to import data from Excel, so that I can batch enter data.</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Upload .xlsx file
-2) Preview imported data
-3) Confirm import</t>
+    <t xml:space="preserve">1. Upload .xlsx file
+2. Preview imported data
+3. Confirm import</t>
   </si>
 </sst>
 </file>
@@ -600,22 +600,22 @@
         <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
         <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H4" t="s">
         <v>17</v>
       </c>
       <c r="I4" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
@@ -623,31 +623,31 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G5" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="H5" t="s">
         <v>17</v>
       </c>
       <c r="I5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="J5" t="s">
         <v>19</v>
@@ -655,13 +655,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
@@ -670,16 +670,16 @@
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G6" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
         <v>17</v>
       </c>
       <c r="I6" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="J6" t="s">
         <v>19</v>
@@ -687,31 +687,31 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H7" t="s">
         <v>17</v>
       </c>
       <c r="I7" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="J7" t="s">
         <v>19</v>
@@ -719,31 +719,31 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="H8" t="s">
         <v>17</v>
       </c>
       <c r="I8" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="J8" t="s">
         <v>19</v>
@@ -751,22 +751,22 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" t="s">
         <v>52</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>53</v>
-      </c>
-      <c r="C9" t="s">
-        <v>54</v>
       </c>
       <c r="D9" t="s">
         <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G9" t="s">
         <v>16</v>
@@ -775,7 +775,7 @@
         <v>17</v>
       </c>
       <c r="I9" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="J9" t="s">
         <v>19</v>
@@ -792,13 +792,13 @@
         <v>58</v>
       </c>
       <c r="D10" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G10" t="s">
         <v>24</v>
@@ -807,7 +807,7 @@
         <v>17</v>
       </c>
       <c r="I10" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="J10" t="s">
         <v>19</v>
@@ -815,31 +815,31 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" t="s">
+        <v>66</v>
+      </c>
+      <c r="G11" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" t="s">
         <v>61</v>
-      </c>
-      <c r="C11" t="s">
-        <v>62</v>
-      </c>
-      <c r="D11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" t="s">
-        <v>48</v>
-      </c>
-      <c r="F11" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" t="s">
-        <v>16</v>
-      </c>
-      <c r="H11" t="s">
-        <v>17</v>
-      </c>
-      <c r="I11" t="s">
-        <v>64</v>
       </c>
       <c r="J11" t="s">
         <v>19</v>
@@ -847,22 +847,22 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D12" t="s">
         <v>13</v>
       </c>
       <c r="E12" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="F12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G12" t="s">
         <v>16</v>
@@ -871,7 +871,7 @@
         <v>17</v>
       </c>
       <c r="I12" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="J12" t="s">
         <v>19</v>
@@ -879,22 +879,22 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D13" t="s">
         <v>13</v>
       </c>
       <c r="E13" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="F13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G13" t="s">
         <v>16</v>
@@ -903,7 +903,7 @@
         <v>17</v>
       </c>
       <c r="I13" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="J13" t="s">
         <v>19</v>
@@ -911,22 +911,22 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D14" t="s">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>14</v>
       </c>
       <c r="F14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G14" t="s">
         <v>24</v>
@@ -935,7 +935,7 @@
         <v>17</v>
       </c>
       <c r="I14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J14" t="s">
         <v>19</v>
@@ -943,31 +943,31 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D15" t="s">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E15" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
       <c r="G15" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="H15" t="s">
         <v>17</v>
       </c>
       <c r="I15" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="J15" t="s">
         <v>19</v>
@@ -984,22 +984,22 @@
         <v>86</v>
       </c>
       <c r="D16" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="E16" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G16" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="H16" t="s">
         <v>17</v>
       </c>
       <c r="I16" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="J16" t="s">
         <v>19</v>
@@ -1007,31 +1007,31 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D17" t="s">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="F17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G17" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="H17" t="s">
         <v>17</v>
       </c>
       <c r="I17" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="J17" t="s">
         <v>19</v>
@@ -1048,10 +1048,10 @@
         <v>96</v>
       </c>
       <c r="D18" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="E18" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F18" t="s">
         <v>97</v>
@@ -1063,7 +1063,7 @@
         <v>17</v>
       </c>
       <c r="I18" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="J18" t="s">
         <v>19</v>
@@ -1083,7 +1083,7 @@
         <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F19" t="s">
         <v>101</v>
@@ -1112,10 +1112,10 @@
         <v>105</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="E20" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F20" t="s">
         <v>106</v>
@@ -1144,10 +1144,10 @@
         <v>109</v>
       </c>
       <c r="D21" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="E21" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F21" t="s">
         <v>110</v>
@@ -1176,7 +1176,7 @@
         <v>113</v>
       </c>
       <c r="D22" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="E22" t="s">
         <v>114</v>
@@ -1208,7 +1208,7 @@
         <v>119</v>
       </c>
       <c r="D23" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="E23" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
fix: v3 — template-exact formatting — Times New Roman, TableGrid, Heading1/2 styles, correct page margins, MoSCoW sprint tables, numbered lists, AC '1.' format, US011 fixed actor
</commit_message>
<xml_diff>
--- a/deliverables/ProductBacklog_group104.xlsx
+++ b/deliverables/ProductBacklog_group104.xlsx
@@ -1,14 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10302"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{65E3B90D-658D-1D4D-95E4-853C40A4EE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="600" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
   <si>
     <t xml:space="preserve">Story ID</t>
   </si>
@@ -40,6 +47,9 @@
     <t xml:space="preserve">Date finished (or planned)</t>
   </si>
   <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
     <t xml:space="preserve">US001</t>
   </si>
   <si>
@@ -55,24 +65,18 @@
     <t xml:space="preserve">Sprint 1</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Can enter email and password
-2. Password strength validation
-3. Success confirmation
-4. Email verification link</t>
+    <t xml:space="preserve">1. Can enter email and password.
+2. Password strength validation.
+3. Success confirmation.
+4. Email verification link.</t>
   </si>
   <si>
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve"/>
-  </si>
-  <si>
     <t xml:space="preserve">2026-04-07</t>
   </si>
   <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
     <t xml:space="preserve">US002</t>
   </si>
   <si>
@@ -82,10 +86,10 @@
     <t xml:space="preserve">As a registered user, I want to log in, so that I can access my data.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Correct credentials allow login
-2. Wrong password shows error
-3. Remember login state
-4. Redirect to home after login</t>
+    <t xml:space="preserve">1. Correct credentials allow login.
+2. Wrong password shows error.
+3. Remember login state.
+4. Redirect to home after login.</t>
   </si>
   <si>
     <t xml:space="preserve">3</t>
@@ -103,9 +107,9 @@
     <t xml:space="preserve">Should</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Enter old and new password
-2. Confirm new password
-3. Success notification</t>
+    <t xml:space="preserve">1. Enter old and new password.
+2. Confirm new password.
+3. Success notification.</t>
   </si>
   <si>
     <t xml:space="preserve">2026-04-10</t>
@@ -123,9 +127,9 @@
     <t xml:space="preserve">Sprint 2</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Assign user roles
-2. View role list
-3. Modify user permissions</t>
+    <t xml:space="preserve">1. Assign user roles.
+2. View role list.
+3. Modify user permissions.</t>
   </si>
   <si>
     <t xml:space="preserve">8</t>
@@ -143,9 +147,9 @@
     <t xml:space="preserve">As a user, I want to log out, so that I can protect my privacy on shared devices.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click logout button
-2. Clear session
-3. Redirect to login page</t>
+    <t xml:space="preserve">1. Click logout button.
+2. Clear session.
+3. Redirect to login page.</t>
   </si>
   <si>
     <t xml:space="preserve">2</t>
@@ -160,9 +164,9 @@
     <t xml:space="preserve">As a user, I want to create new data records, so that I can manage my information.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Fill in form fields
-2. Save success notification
-3. Auto-generate ID</t>
+    <t xml:space="preserve">1. Fill in form fields.
+2. Save success notification.
+3. Auto-generate ID.</t>
   </si>
   <si>
     <t xml:space="preserve">US007</t>
@@ -174,9 +178,9 @@
     <t xml:space="preserve">As a user, I want to view existing records, so that I can understand the current status.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. List all records
-2. Click to view details
-3. Pagination</t>
+    <t xml:space="preserve">1. List all records.
+2. Click to view details.
+3. Pagination.</t>
   </si>
   <si>
     <t xml:space="preserve">US008</t>
@@ -188,9 +192,9 @@
     <t xml:space="preserve">As a user, I want to edit existing records, so that I can update information.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Modify form fields
-2. Save update
-3. Version tracking</t>
+    <t xml:space="preserve">1. Modify form fields.
+2. Save update.
+3. Version tracking.</t>
   </si>
   <si>
     <t xml:space="preserve">2026-04-16</t>
@@ -208,9 +212,9 @@
     <t xml:space="preserve">Sprint 3</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Confirmation prompt
-2. Soft delete (recoverable)
-3. Permanent delete option</t>
+    <t xml:space="preserve">1. Confirmation prompt.
+2. Soft delete (recoverable).
+3. Permanent delete option.</t>
   </si>
   <si>
     <t xml:space="preserve">2026-04-21</t>
@@ -228,9 +232,9 @@
     <t xml:space="preserve">Could</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Select multiple records
-2. Batch delete/edit/export
-3. Operation confirmation</t>
+    <t xml:space="preserve">1. Select multiple records.
+2. Batch delete/edit/export.
+3. Operation confirmation.</t>
   </si>
   <si>
     <t xml:space="preserve">US011</t>
@@ -242,9 +246,9 @@
     <t xml:space="preserve">As an administrator, I want the system to validate input data, so that I can ensure data quality and prevent errors.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Required field check
-2. Format validation
-3. Uniqueness check</t>
+    <t xml:space="preserve">1. Required field check.
+2. Format validation.
+3. Uniqueness check.</t>
   </si>
   <si>
     <t xml:space="preserve">US012</t>
@@ -256,9 +260,9 @@
     <t xml:space="preserve">As a system, I want to permanently store data, so that users can access it next time.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Database storage
-2. No data loss
-3. Backup support</t>
+    <t xml:space="preserve">1. File-based storage (JSON/XML).
+2. No data loss on restart.
+3. Backup support.</t>
   </si>
   <si>
     <t xml:space="preserve">US013</t>
@@ -270,9 +274,9 @@
     <t xml:space="preserve">As a user, I want to browse the system via navigation menu, so that I can quickly find features.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Sidebar navigation
-2. Current page highlighted
-3. Responsive menu</t>
+    <t xml:space="preserve">1. Sidebar navigation.
+2. Current page highlighted.
+3. Responsive menu.</t>
   </si>
   <si>
     <t xml:space="preserve">2026-04-09</t>
@@ -287,9 +291,9 @@
     <t xml:space="preserve">As a user, I want to see overview data on a dashboard, so that I can quickly understand the status.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Statistics display
-2. Chart visualisation
-3. Quick action entry points</t>
+    <t xml:space="preserve">1. Statistics display.
+2. Chart visualisation.
+3. Quick action entry points.</t>
   </si>
   <si>
     <t xml:space="preserve">US015</t>
@@ -304,9 +308,9 @@
     <t xml:space="preserve">Sprint 4</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Adapt to mobile screens
-2. Touch operation support
-3. Fast loading</t>
+    <t xml:space="preserve">1. Adapt to mobile screens.
+2. Touch operation support.
+3. Fast loading.</t>
   </si>
   <si>
     <t xml:space="preserve">2026-04-28</t>
@@ -321,9 +325,9 @@
     <t xml:space="preserve">As a user, I want to fill in clear forms, so that I can efficiently input data.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Clear labels
-2. Input hint text
-3. Real-time validation feedback</t>
+    <t xml:space="preserve">1. Clear labels.
+2. Input hint text.
+3. Real-time validation feedback.</t>
   </si>
   <si>
     <t xml:space="preserve">US017</t>
@@ -335,9 +339,9 @@
     <t xml:space="preserve">As a user, I want to receive operation feedback notifications, so that I can understand system status.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Success/failure prompts
-2. Toast messages
-3. Dismissable notifications</t>
+    <t xml:space="preserve">1. Success/failure prompts.
+2. Toast messages.
+3. Dismissable notifications.</t>
   </si>
   <si>
     <t xml:space="preserve">US018</t>
@@ -349,9 +353,9 @@
     <t xml:space="preserve">As a user, I want to search records, so that I can quickly find target data.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Keyword search input
-2. Highlight matching results
-3. Search history</t>
+    <t xml:space="preserve">1. Keyword search input.
+2. Highlight matching results.
+3. Search history.</t>
   </si>
   <si>
     <t xml:space="preserve">2026-05-05</t>
@@ -366,9 +370,9 @@
     <t xml:space="preserve">As a user, I want to filter data by conditions, so that I can precisely select.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Multiple condition combination
-2. Date range filter
-3. Status filter</t>
+    <t xml:space="preserve">1. Multiple condition combination.
+2. Date range filter.
+3. Status filter.</t>
   </si>
   <si>
     <t xml:space="preserve">US020</t>
@@ -380,9 +384,9 @@
     <t xml:space="preserve">As a user, I want to sort records, so that I can view them by priority.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Sort by date
-2. Sort by name
-3. Sort by priority</t>
+    <t xml:space="preserve">1. Sort by date.
+2. Sort by name.
+3. Sort by priority.</t>
   </si>
   <si>
     <t xml:space="preserve">US021</t>
@@ -397,9 +401,9 @@
     <t xml:space="preserve">Sprint 5</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Select export fields
-2. Generate .xlsx file
-3. Auto-download</t>
+    <t xml:space="preserve">1. Select export fields.
+2. Generate .xlsx file.
+3. Auto-download.</t>
   </si>
   <si>
     <t xml:space="preserve">2026-05-12</t>
@@ -414,28 +418,29 @@
     <t xml:space="preserve">As an administrator, I want to import data from Excel, so that I can batch enter data.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Upload .xlsx file
-2. Preview imported data
-3. Confirm import</t>
+    <t xml:space="preserve">1. Upload .xlsx file.
+2. Preview imported data.
+3. Confirm import.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -447,7 +452,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
@@ -461,37 +467,350 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <!-- 0: Normal -->
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <!-- 1: Header (bold, blue fill, white text) -->
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <!-- 2: Alternating row -->
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
+  <cellStyles count="2">
+    <cellStyle name="40% - Accent1" xfId="1" builtinId="31"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+  <a:themeElements>
+    <a:clrScheme name="Office 2007 - 2010">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office 2007 - 2010">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office 2007 - 2010">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A23"/>
+  <col xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" min="1" max="1" width="9.1640625" style="1" customWidth="1"/>
+  <col xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" min="2" max="2" width="16.6640625" style="1" customWidth="1"/>
+  <col xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" min="3" max="3" width="36" style="1" customWidth="1"/>
+  <col xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" min="4" max="4" width="9.1640625" style="1"/>
+  <col xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" min="5" max="5" width="28.33203125" style="1" customWidth="1"/>
+  <col xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" min="6" max="7" width="19.83203125" style="1" customWidth="1"/>
+  <col xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" min="8" max="8" width="17.1640625" style="1" customWidth="1"/>
+  <col xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" min="9" max="9" width="24.83203125" style="1" customWidth="1"/>
+  <col xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" min="10" max="10" width="26.33203125" style="1" customWidth="1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
@@ -527,706 +846,706 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I2" t="s">
         <v>18</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
         <v>20</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>23</v>
       </c>
-      <c r="G3" t="s">
-        <v>24</v>
-      </c>
       <c r="H3" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I3" t="s">
         <v>18</v>
       </c>
       <c r="J3" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" t="s">
         <v>29</v>
       </c>
-      <c r="G4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" t="s">
-        <v>30</v>
-      </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
         <v>31</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>32</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" t="s">
         <v>33</v>
       </c>
-      <c r="D5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>34</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>35</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" t="s">
         <v>36</v>
       </c>
-      <c r="H5" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" t="s">
-        <v>37</v>
-      </c>
       <c r="J5" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
         <v>38</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>39</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" t="s">
         <v>40</v>
       </c>
-      <c r="D6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>41</v>
       </c>
-      <c r="G6" t="s">
-        <v>42</v>
-      </c>
       <c r="H6" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I6" t="s">
         <v>18</v>
       </c>
       <c r="J6" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>44</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" t="s">
         <v>45</v>
       </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" t="s">
-        <v>46</v>
-      </c>
       <c r="G7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H7" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J7" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
         <v>47</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>48</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" t="s">
         <v>49</v>
       </c>
-      <c r="D8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" t="s">
-        <v>50</v>
-      </c>
       <c r="G8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H8" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J8" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s">
         <v>51</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>52</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" t="s">
         <v>53</v>
       </c>
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" t="s">
+        <v>10</v>
+      </c>
+      <c r="I9" t="s">
         <v>54</v>
       </c>
-      <c r="G9" t="s">
-        <v>16</v>
-      </c>
-      <c r="H9" t="s">
-        <v>17</v>
-      </c>
-      <c r="I9" t="s">
-        <v>55</v>
-      </c>
       <c r="J9" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
         <v>56</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>57</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" t="s">
         <v>58</v>
       </c>
-      <c r="D10" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>59</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10" t="s">
+        <v>10</v>
+      </c>
+      <c r="I10" t="s">
         <v>60</v>
       </c>
-      <c r="G10" t="s">
-        <v>24</v>
-      </c>
-      <c r="H10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I10" t="s">
-        <v>61</v>
-      </c>
       <c r="J10" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
         <v>62</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>63</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>64</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" t="s">
         <v>65</v>
       </c>
-      <c r="E11" t="s">
-        <v>59</v>
-      </c>
-      <c r="F11" t="s">
-        <v>66</v>
-      </c>
       <c r="G11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H11" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J11" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
         <v>67</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>68</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" t="s">
         <v>69</v>
       </c>
-      <c r="D12" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" t="s">
-        <v>34</v>
-      </c>
-      <c r="F12" t="s">
-        <v>70</v>
-      </c>
       <c r="G12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H12" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J12" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
         <v>71</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>72</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" t="s">
         <v>73</v>
       </c>
-      <c r="D13" t="s">
-        <v>13</v>
-      </c>
-      <c r="E13" t="s">
-        <v>34</v>
-      </c>
-      <c r="F13" t="s">
-        <v>74</v>
-      </c>
       <c r="G13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H13" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J13" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" t="s">
         <v>75</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>76</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" t="s">
         <v>77</v>
       </c>
-      <c r="D14" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
+        <v>23</v>
+      </c>
+      <c r="H14" t="s">
+        <v>10</v>
+      </c>
+      <c r="I14" t="s">
         <v>78</v>
       </c>
-      <c r="G14" t="s">
-        <v>24</v>
-      </c>
-      <c r="H14" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" t="s">
-        <v>79</v>
-      </c>
       <c r="J14" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" t="s">
         <v>80</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>81</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" t="s">
         <v>82</v>
       </c>
-      <c r="D15" t="s">
-        <v>28</v>
-      </c>
-      <c r="E15" t="s">
-        <v>59</v>
-      </c>
-      <c r="F15" t="s">
-        <v>83</v>
-      </c>
       <c r="G15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H15" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J15" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" t="s">
         <v>84</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>85</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" t="s">
         <v>86</v>
       </c>
-      <c r="D16" t="s">
-        <v>28</v>
-      </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>87</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" t="s">
+        <v>10</v>
+      </c>
+      <c r="I16" t="s">
         <v>88</v>
       </c>
-      <c r="G16" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" t="s">
-        <v>89</v>
-      </c>
       <c r="J16" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" t="s">
         <v>90</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>91</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s">
         <v>92</v>
       </c>
-      <c r="D17" t="s">
-        <v>13</v>
-      </c>
-      <c r="E17" t="s">
-        <v>14</v>
-      </c>
-      <c r="F17" t="s">
-        <v>93</v>
-      </c>
       <c r="G17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H17" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J17" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" t="s">
         <v>94</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>95</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" t="s">
+        <v>86</v>
+      </c>
+      <c r="F18" t="s">
         <v>96</v>
       </c>
-      <c r="D18" t="s">
-        <v>65</v>
-      </c>
-      <c r="E18" t="s">
-        <v>87</v>
-      </c>
-      <c r="F18" t="s">
-        <v>97</v>
-      </c>
       <c r="G18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H18" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J18" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
+        <v>97</v>
+      </c>
+      <c r="B19" t="s">
         <v>98</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>99</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" t="s">
+        <v>86</v>
+      </c>
+      <c r="F19" t="s">
         <v>100</v>
       </c>
-      <c r="D19" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" t="s">
-        <v>87</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" t="s">
         <v>101</v>
       </c>
-      <c r="G19" t="s">
-        <v>16</v>
-      </c>
-      <c r="H19" t="s">
-        <v>17</v>
-      </c>
-      <c r="I19" t="s">
-        <v>102</v>
-      </c>
       <c r="J19" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" t="s">
         <v>103</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>104</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" t="s">
         <v>105</v>
       </c>
-      <c r="D20" t="s">
-        <v>28</v>
-      </c>
-      <c r="E20" t="s">
-        <v>87</v>
-      </c>
-      <c r="F20" t="s">
-        <v>106</v>
-      </c>
       <c r="G20" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H20" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I20" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J20" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" t="s">
         <v>107</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>108</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" t="s">
+        <v>86</v>
+      </c>
+      <c r="F21" t="s">
         <v>109</v>
       </c>
-      <c r="D21" t="s">
-        <v>65</v>
-      </c>
-      <c r="E21" t="s">
-        <v>87</v>
-      </c>
-      <c r="F21" t="s">
-        <v>110</v>
-      </c>
       <c r="G21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H21" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I21" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J21" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B22" t="s">
         <v>111</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>112</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" t="s">
         <v>113</v>
       </c>
-      <c r="D22" t="s">
-        <v>28</v>
-      </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>114</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" t="s">
+        <v>10</v>
+      </c>
+      <c r="I22" t="s">
         <v>115</v>
       </c>
-      <c r="G22" t="s">
-        <v>16</v>
-      </c>
-      <c r="H22" t="s">
-        <v>17</v>
-      </c>
-      <c r="I22" t="s">
-        <v>116</v>
-      </c>
       <c r="J22" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>116</v>
+      </c>
+      <c r="B23" t="s">
         <v>117</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>118</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
+        <v>64</v>
+      </c>
+      <c r="E23" t="s">
+        <v>113</v>
+      </c>
+      <c r="F23" t="s">
         <v>119</v>
       </c>
-      <c r="D23" t="s">
-        <v>65</v>
-      </c>
-      <c r="E23" t="s">
-        <v>114</v>
-      </c>
-      <c r="F23" t="s">
-        <v>120</v>
-      </c>
       <c r="G23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H23" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="I23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J23" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>